<commit_message>
Add multi-sheet marker support and one-click toolbar
- Метки вида {Лист!A5} читают ячейку с указанного листа книги;
  {A5} по-прежнему берёт лист по умолчанию из настроек
- Кириллица проверяется только в адресе (русские имена листов допустимы)
- Автосоздание панели SmartCells на вкладке «Надстройки» с кнопками
  Обновить/Настройки/Убрать связь — ручная настройка QAT больше не нужна
- Тестовые файлы: добавлен второй лист и метка {Лист2!A1}
- Обновлены INSTALL.md и TEST_PLAN.md

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoXxRKY7BcWh69G1JzSWJ6
</commit_message>
<xml_diff>
--- a/test/Тест_данные.xlsx
+++ b/test/Тест_данные.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Данные" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лист2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,4 +503,25 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Значение со второго листа</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix packaging: CRLF line endings, .gitattributes, Excel format codes
- src/*.bas и src/*.cls переведены на CRLF — редактор VBA на Windows
  некорректно импортирует файлы с Unix-окончаниями строк
- .gitattributes: запрет нормализации VBA-файлов git-ом, чтобы cp1251+CRLF
  доходили до пользователя байт-в-байт (включая Download ZIP)
- make_test_files.py: формат-коды чисел приведены к en-US синтаксису
  ('#,##0.00') — Excel хранит коды именно так, отображая по локали;
  тестовые файлы перегенерированы

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoXxRKY7BcWh69G1JzSWJ6
</commit_message>
<xml_diff>
--- a/test/Тест_данные.xlsx
+++ b/test/Тест_данные.xlsx
@@ -17,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="# ##0,00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +53,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>